<commit_message>
docs(aisan_lbo_case): external-facing wording in Excel + slide hedging + log accuracy
- Excel: Assumptions!B5 "post-fraud-news" -> "post-investigation disclosure";
  Scenarios!G7 drop internal "treasury-share correction" narrative (recalc
  446 formulas, 0 errors, values unchanged).
- PPTX: prefix standalone "forgery & concealment" with "suspected" on slides
  2 and 18 (match the cautious FACT_CHECK framing).
- Docs: fix remaining current-state "19 slides" -> 20 (HANDOFF §9, FACT_CHECK);
  dated round logs kept as historical record.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aisan_lbo_case/docs/AISAN_4667_LBO_Model.xlsx
+++ b/aisan_lbo_case/docs/AISAN_4667_LBO_Model.xlsx
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Financing structure</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference share price (¥, post-fraud-news)</t>
+    <t xml:space="preserve">Reference share price (¥, post-investigation disclosure)</t>
   </si>
   <si>
     <t xml:space="preserve">5-Jun-26 close</t>
@@ -789,7 +789,7 @@
     <t xml:space="preserve">Exit EBITDA (¥mm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Base: mid-single-digit growth, gradual margin lift to 12% via mix &amp; cost discipline; exit 10x. Returns improve after treasury-share correction but remain below a clean 20% hurdle.</t>
+    <t xml:space="preserve">Base: mid-single-digit growth, gradual margin lift to 12% via mix &amp; cost discipline; exit 10x; returns remain below a clean 20% hurdle.</t>
   </si>
   <si>
     <t xml:space="preserve">Exit EV/EBITDA</t>

</xml_diff>